<commit_message>
Actualización del archivo de casos de prueba de NeuroClerk
</commit_message>
<xml_diff>
--- a/casos_de_prueba_NeuroClerk.xlsx
+++ b/casos_de_prueba_NeuroClerk.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="144">
   <si>
     <t xml:space="preserve">Casos de prueba de NeuroClerk (probar_rag.py)</t>
   </si>
@@ -30,7 +30,7 @@
     <t xml:space="preserve">Cómo usarla: las columnas grises describen cada caso y salen de probar_rag.py. Completa las columnas amarillas (Tabla, Fuente, Respuesta) con OK, FALLA o ERROR después de correr 'python probar_rag.py --llm'. 'N/A' cuando el caso no mide esa columna.</t>
   </si>
   <si>
-    <t xml:space="preserve">Resultados: línea de base del 27/10/2026, 59 documentos, proveedor Gemini.</t>
+    <t xml:space="preserve">Resultados: ejecución del 27/10/2026 con límite de 2 fragmentos por página, 59 documentos, gemini-3.5-flash-lite.</t>
   </si>
   <si>
     <t xml:space="preserve">N.º</t>
@@ -90,7 +90,7 @@
     <t xml:space="preserve">OK</t>
   </si>
   <si>
-    <t xml:space="preserve">Tabla en el puesto 1 (0.909). Nombra fármacos que solo están en la tabla.</t>
+    <t xml:space="preserve">Tabla en el puesto 1 (0.909).</t>
   </si>
   <si>
     <t xml:space="preserve">¿Qué fármacos pueden causar síndrome serotoninérgico?</t>
@@ -114,7 +114,7 @@
     <t xml:space="preserve">Menciona alguna de: ebastina, retigabina, piperaquina, eribulina</t>
   </si>
   <si>
-    <t xml:space="preserve">Tabla en el puesto 5 (0.881).</t>
+    <t xml:space="preserve">Tabla en el puesto 5; nombra ebastina, retigabina y eribulina.</t>
   </si>
   <si>
     <t xml:space="preserve">¿Qué interacción tienen los IECA con el litio?</t>
@@ -129,7 +129,7 @@
     <t xml:space="preserve">Menciona alguna de: toxicidad, concentraci, nivel</t>
   </si>
   <si>
-    <t xml:space="preserve">Tabla en el puesto 1; fue el único fragmento que pasó el filtro.</t>
+    <t xml:space="preserve">Tabla en el puesto 1; único fragmento que pasó el filtro.</t>
   </si>
   <si>
     <t xml:space="preserve">¿Qué isoenzimas del citocromo P450 metabolizan la clozapina?</t>
@@ -144,7 +144,7 @@
     <t xml:space="preserve">Menciona alguna de: cyp1a2, 1a2</t>
   </si>
   <si>
-    <t xml:space="preserve">Tabla en el puesto 1, pero cinco filas de la Tabla 2 (pág. 254) ocupan el contexto.</t>
+    <t xml:space="preserve">Tabla en el puesto 1. Con el límite por página, la Tabla 2 aporta 2 filas en vez de 5.</t>
   </si>
   <si>
     <t xml:space="preserve">¿Cómo se metaboliza el alprazolam?</t>
@@ -171,7 +171,7 @@
     <t xml:space="preserve">Menciona alguna de: imatinib, pazopanib, cinacalcet</t>
   </si>
   <si>
-    <t xml:space="preserve">Tabla en el puesto 9 de 10: entra justo.</t>
+    <t xml:space="preserve">Tabla en el puesto 9 de 10. El límite por página corta la continuación de la Tabla 6.</t>
   </si>
   <si>
     <t xml:space="preserve">Ficha: dosis</t>
@@ -204,61 +204,61 @@
     <t xml:space="preserve">FT_Clozapina.pdf</t>
   </si>
   <si>
-    <t xml:space="preserve">Menciona alguna de: neutrofilos, leucocitos</t>
+    <t xml:space="preserve">Menciona alguna de: neutrofilos, leucocitos, ran, recuento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mejoró por la corrección de la prueba: ahora acepta 'RAN'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ficha: niveles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Qué concentraciones de litio en sangre se consideran terapéuticas?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FT_Litio.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona alguna de: meq, mmol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona mEq.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diagnóstico (DSM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Cuánto tiempo deben durar los síntomas para diagnosticar un episodio de depresión mayor?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DSM-5-TR.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona alguna de: dos semanas, 2 semanas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DSM pág. 213 en el puesto 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diagnóstico (CIE-11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En la nueva clasificación, ¿en qué agrupación quedaron la esquizofrenia y los trastornos delirantes de la CIE-10?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIE-11.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona alguna de: 6a20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVISO: ninguna clave aparece en su fuente</t>
   </si>
   <si>
     <t xml:space="preserve">FALLA</t>
   </si>
   <si>
-    <t xml:space="preserve">Fallo de la prueba: la ficha usa la sigla RAN. Agregar 'ran' y 'recuento' a las claves.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ficha: niveles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">¿Qué concentraciones de litio en sangre se consideran terapéuticas?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FT_Litio.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona alguna de: meq, mmol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona mEq.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diagnóstico (DSM)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">¿Cuánto tiempo deben durar los síntomas para diagnosticar un episodio de depresión mayor?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DSM-5-TR.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona alguna de: dos semanas, 2 semanas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DSM pág. 213 en el puesto 1; menciona 'dos semanas'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diagnóstico (CIE-11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">¿Qué código tiene la esquizofrenia en la clasificación internacional de enfermedades?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIE-11.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona alguna de: 6a20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVISO: ninguna clave aparece en su fuente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caso mal armado: '6a20' no está en la guía de referencia de la CIE-11. Reemplazar la pregunta. El modelo respondió que el contexto no alcanzaba.</t>
+    <t xml:space="preserve">Pregunta del bloque F20-F29: llegan págs. 503-528 de la CIE-11, pero la 504 (la equivalencia) queda 7.ª y el modelo dijo que no había información. Pregunta reformulada sin el código para la próxima ejecución.</t>
   </si>
   <si>
     <t xml:space="preserve">Guía (mhGAP)</t>
@@ -273,7 +273,7 @@
     <t xml:space="preserve">Menciona alguna de: fluoxetina, amitriptilina</t>
   </si>
   <si>
-    <t xml:space="preserve">Fallo real: siete filas de la Tabla 1 del libro coparon el contexto; el Cuadro 1 de la mhGAP llegó 9.º y 10.º.</t>
+    <t xml:space="preserve">El filtro de duplicados no cambió nada: los dos fragmentos de la pág. 34 son textos distintos. La pág. 36 queda en el puesto 11 con tope 10. Se sube MAX_FRAGMENTOS a 12.</t>
   </si>
   <si>
     <t xml:space="preserve">Formulario (MSP)</t>
@@ -288,7 +288,7 @@
     <t xml:space="preserve">Menciona alguna de: haloperidol, risperidona</t>
   </si>
   <si>
-    <t xml:space="preserve">Fallo real: filas de tablas del libro coparon el contexto; del Formulario solo llegó la portada.</t>
+    <t xml:space="preserve">Nombra haloperidol y risperidona.</t>
   </si>
   <si>
     <t xml:space="preserve">CYP (Flockhart)</t>
@@ -303,7 +303,7 @@
     <t xml:space="preserve">Menciona alguna de: rifampicina, rifampin, carbamazepina, carbamazepine</t>
   </si>
   <si>
-    <t xml:space="preserve">Respondió desde la Tabla 8 del libro; la tabla de Flockhart no apareció.</t>
+    <t xml:space="preserve">Respondió desde la Tabla 8 del libro; la tabla de Flockhart sigue sin aparecer.</t>
   </si>
   <si>
     <t xml:space="preserve">Escala</t>
@@ -318,7 +318,7 @@
     <t xml:space="preserve">Menciona alguna de: 27</t>
   </si>
   <si>
-    <t xml:space="preserve">Llegó un solo fragmento del PHQ-9; el modelo dijo que no tenía el puntaje máximo.</t>
+    <t xml:space="preserve">Llega un solo fragmento del PHQ-9, sin el puntaje máximo. Revisar con --buscar 27 PHQ-9_Spanish.pdf.</t>
   </si>
   <si>
     <t xml:space="preserve">Caso clínico</t>
@@ -333,7 +333,7 @@
     <t xml:space="preserve">Menciona alguna de: 1a2, aument</t>
   </si>
   <si>
-    <t xml:space="preserve">Ficha de clozapina en el puesto 1; menciona CYP1A2.</t>
+    <t xml:space="preserve">Respuesta correcta ('se elimina el efecto inductor del tabaco... reducir las dosis'), pero sin '1a2' ni 'aument'. Se agregan 'inductor' y 'reduc' a las claves.</t>
   </si>
   <si>
     <t xml:space="preserve">Sin respuesta</t>
@@ -423,7 +423,7 @@
     <t xml:space="preserve">Línea de base: tablas por filas y categorías, cupo proporcional, 59 documentos</t>
   </si>
   <si>
-    <t xml:space="preserve">Gemini (anotar si fue 3.8-flash o 3.5-flash-lite)</t>
+    <t xml:space="preserve">Gemini (modelo no anotado)</t>
   </si>
   <si>
     <t xml:space="preserve">7/7</t>
@@ -436,6 +436,24 @@
   </si>
   <si>
     <t xml:space="preserve">2/2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Límite de 2 fragmentos por página; caso 9 acepta 'RAN'; pausa y reintentos en las pruebas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gemini-3.5-flash-lite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14/17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtro de casi duplicados (SIMILITUD_DUPLICADO 0.5); caso 12 reemplazado por el bloque F20-F29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17/17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13/17</t>
   </si>
 </sst>
 </file>
@@ -573,7 +591,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -590,7 +608,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -627,18 +645,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -946,7 +952,7 @@
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -1325,10 +1331,10 @@
         <v>21</v>
       </c>
       <c r="K13" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="L13" s="7" t="s">
         <v>61</v>
-      </c>
-      <c r="L13" s="7" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1336,22 +1342,22 @@
         <v>10</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E14" s="7" t="s">
         <v>64</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>65</v>
       </c>
       <c r="F14" s="7" t="s">
         <v>53</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H14" s="7" t="s">
         <v>20</v>
@@ -1366,7 +1372,7 @@
         <v>21</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1374,22 +1380,22 @@
         <v>11</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="E15" s="7" t="s">
         <v>69</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>70</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>53</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H15" s="7" t="s">
         <v>20</v>
@@ -1404,7 +1410,7 @@
         <v>21</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1412,34 +1418,34 @@
         <v>12</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E16" s="7" t="s">
         <v>74</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>75</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>53</v>
       </c>
       <c r="G16" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="H16" s="7" t="s">
         <v>76</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>77</v>
       </c>
       <c r="I16" s="7" t="s">
         <v>55</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="L16" s="7" t="s">
         <v>78</v>
@@ -1477,7 +1483,7 @@
         <v>21</v>
       </c>
       <c r="K17" s="8" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="L17" s="7" t="s">
         <v>83</v>
@@ -1515,7 +1521,7 @@
         <v>21</v>
       </c>
       <c r="K18" s="8" t="s">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="L18" s="7" t="s">
         <v>88</v>
@@ -1591,7 +1597,7 @@
         <v>21</v>
       </c>
       <c r="K20" s="8" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="L20" s="7" t="s">
         <v>98</v>
@@ -1629,7 +1635,7 @@
         <v>21</v>
       </c>
       <c r="K21" s="8" t="s">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="L21" s="7" t="s">
         <v>103</v>
@@ -1807,7 +1813,7 @@
       </c>
       <c r="B6" s="11" t="n">
         <f aca="false">COUNTIF(Casos!J5:J23,"OK")</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C6" s="11" t="n">
         <f aca="false">COUNTIF(Casos!J5:J23,"OK")+COUNTIF(Casos!J5:J23,"FALLA")</f>
@@ -1815,7 +1821,7 @@
       </c>
       <c r="D6" s="12" t="n">
         <f aca="false">IF(C6=0,"-",B6/C6)</f>
-        <v>0.941176470588235</v>
+        <v>1</v>
       </c>
       <c r="E6" s="11" t="s">
         <v>121</v>
@@ -1827,7 +1833,7 @@
       </c>
       <c r="B7" s="11" t="n">
         <f aca="false">COUNTIF(Casos!K5:K23,"OK")</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C7" s="11" t="n">
         <f aca="false">COUNTIF(Casos!K5:K23,"OK")+COUNTIF(Casos!K5:K23,"FALLA")</f>
@@ -1835,7 +1841,7 @@
       </c>
       <c r="D7" s="12" t="n">
         <f aca="false">IF(C7=0,"-",B7/C7)</f>
-        <v>0.736842105263158</v>
+        <v>0.789473684210526</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>123</v>
@@ -1866,55 +1872,55 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="15" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="9" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="10" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
         <v>131</v>
       </c>
@@ -1937,6 +1943,54 @@
         <v>137</v>
       </c>
       <c r="H5" s="8"/>
+    </row>
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="H6" s="8"/>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="H7" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>